<commit_message>
estimate lapse sinchai, lama bisauna meldanda bisrame sadak and valuation bhimsen mandir given
</commit_message>
<xml_diff>
--- a/2083_2084/estimate/budget maag estimate/lapse sinchai/for prbn.xlsx
+++ b/2083_2084/estimate/budget maag estimate/lapse sinchai/for prbn.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\2083_2084\estimate\budget maag estimate\lapse sinchai\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\2083_2084\estimate\budget maag estimate\lapse sinchai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F058DA-79A5-4B0F-8475-35F12834D2D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D30DCE20-48D9-42F7-B1C7-CCBB949BDD04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WCR" sheetId="27" state="hidden" r:id="rId1"/>
@@ -491,6 +491,24 @@
     <t>F.Y.:-2083/084</t>
   </si>
   <si>
+    <t>husf] vf8ndf 9'+uf eg]{ / n]en ug]{ sfddf</t>
+  </si>
+  <si>
+    <t>-for column</t>
+  </si>
+  <si>
+    <t>-stirrups</t>
+  </si>
+  <si>
+    <t>Provisional sum for unforseen works of water tank and lab tests</t>
+  </si>
+  <si>
+    <t>-floor</t>
+  </si>
+  <si>
+    <t>g/d k|sf/sf] Sn] / l;N6L df6f]df ;j} lsl;dsf] vGg] sfd</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="14"/>
@@ -506,29 +524,11 @@
         <color theme="1"/>
         <rFont val="Preeti"/>
       </rPr>
-      <t>k+rkfn] If]qdf l;FrfO 6ØfÍL</t>
+      <t>nK;] l;FrfO of]hgf lgdf{0f</t>
     </r>
   </si>
   <si>
-    <t>Date: 2082/06/14</t>
-  </si>
-  <si>
-    <t>husf] vf8ndf 9'+uf eg]{ / n]en ug]{ sfddf</t>
-  </si>
-  <si>
-    <t>-for column</t>
-  </si>
-  <si>
-    <t>-stirrups</t>
-  </si>
-  <si>
-    <t>Provisional sum for unforseen works of water tank and lab tests</t>
-  </si>
-  <si>
-    <t>-floor</t>
-  </si>
-  <si>
-    <t>g/d k|sf/sf] Sn] / l;N6L df6f]df ;j} lsl;dsf] vGg] sfd</t>
+    <t>Date: 2082/06/26</t>
   </si>
 </sst>
 </file>
@@ -536,28 +536,28 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="22">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="#."/>
-    <numFmt numFmtId="169" formatCode="0.00_)"/>
-    <numFmt numFmtId="170" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="171" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="172" formatCode="_ * #,##0_)&quot;$&quot;_ ;_ * \(#,##0\)&quot;$&quot;_ ;_ * &quot;-&quot;_)&quot;$&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="173" formatCode="General_)"/>
-    <numFmt numFmtId="174" formatCode="_ * #,##0_)_$_ ;_ * \(#,##0\)_$_ ;_ * &quot;-&quot;_)_$_ ;_ @_ "/>
-    <numFmt numFmtId="175" formatCode="_ * #,##0.00_)&quot;$&quot;_ ;_ * \(#,##0.00\)&quot;$&quot;_ ;_ * &quot;-&quot;??_)&quot;$&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_)_$_ ;_ * \(#,##0.00\)_$_ ;_ * &quot;-&quot;??_)_$_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="mmmm\ d\,\ yyyy"/>
-    <numFmt numFmtId="178" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#.##0\)"/>
-    <numFmt numFmtId="179" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="180" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="181" formatCode="_ &quot;\&quot;* #,##0_ ;_ &quot;\&quot;* \-#,##0_ ;_ &quot;\&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="182" formatCode="_ &quot;\&quot;* #,##0.00_ ;_ &quot;\&quot;* \-#,##0.00_ ;_ &quot;\&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="183" formatCode="0.0"/>
-    <numFmt numFmtId="184" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="5" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="#."/>
+    <numFmt numFmtId="168" formatCode="0.00_)"/>
+    <numFmt numFmtId="169" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="170" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="171" formatCode="_ * #,##0_)&quot;$&quot;_ ;_ * \(#,##0\)&quot;$&quot;_ ;_ * &quot;-&quot;_)&quot;$&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="172" formatCode="General_)"/>
+    <numFmt numFmtId="173" formatCode="_ * #,##0_)_$_ ;_ * \(#,##0\)_$_ ;_ * &quot;-&quot;_)_$_ ;_ @_ "/>
+    <numFmt numFmtId="174" formatCode="_ * #,##0.00_)&quot;$&quot;_ ;_ * \(#,##0.00\)&quot;$&quot;_ ;_ * &quot;-&quot;??_)&quot;$&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="175" formatCode="_ * #,##0.00_)_$_ ;_ * \(#,##0.00\)_$_ ;_ * &quot;-&quot;??_)_$_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="mmmm\ d\,\ yyyy"/>
+    <numFmt numFmtId="177" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#.##0\)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="180" formatCode="_ &quot;\&quot;* #,##0_ ;_ &quot;\&quot;* \-#,##0_ ;_ &quot;\&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="181" formatCode="_ &quot;\&quot;* #,##0.00_ ;_ &quot;\&quot;* \-#,##0.00_ ;_ &quot;\&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="182" formatCode="0.0"/>
+    <numFmt numFmtId="183" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="80">
     <font>
@@ -1589,7 +1589,7 @@
   </borders>
   <cellStyleXfs count="804">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1617,35 +1617,35 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="21" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="22" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="0">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="0">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="0">
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="0">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="0">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="0">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="0">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
@@ -1671,7 +1671,7 @@
     <xf numFmtId="10" fontId="5" fillId="24" borderId="1" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="169" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="168" fontId="30" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
@@ -1720,10 +1720,10 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="28" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
@@ -2092,41 +2092,41 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="170" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyNumberFormat="0" applyFont="0">
       <alignment horizontal="center" vertical="justify"/>
     </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="173" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="167" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="172" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="166" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="173" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf numFmtId="174" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf numFmtId="175" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="173" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="28" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="28" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="28" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="172" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="28" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="28" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="28" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0"/>
-    <xf numFmtId="173" fontId="36" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="172" fontId="36" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="5" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="15"/>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="14" fontId="34" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf numFmtId="38" fontId="29" fillId="0" borderId="16">
       <alignment vertical="center"/>
@@ -2140,11 +2140,11 @@
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="173" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="173" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="172" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="175" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="172" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
@@ -2174,12 +2174,12 @@
     </xf>
     <xf numFmtId="0" fontId="45" fillId="29" borderId="15"/>
     <xf numFmtId="0" fontId="45" fillId="27" borderId="15"/>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="173" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="173" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="172" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="175" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="172" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -2223,10 +2223,10 @@
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="9" fontId="47" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="178" fontId="47" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="179" fontId="47" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="180" fontId="47" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="181" fontId="47" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="47" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="26" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="23" fillId="21" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
@@ -2375,79 +2375,79 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="53" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="53" fillId="0" borderId="0"/>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="0"/>
-    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="55" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="55" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="55" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="56" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="56" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="56" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="53" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="160">
@@ -2471,24 +2471,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="63" fillId="32" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="63" fillId="32" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="63" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="63" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="63" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="63" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="63" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="48" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="48" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="64" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -2532,7 +2532,7 @@
     <xf numFmtId="0" fontId="64" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="65" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2596,12 +2596,12 @@
     <xf numFmtId="0" fontId="65" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="50" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="49" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="50" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="49" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="49" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="49" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="49" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2610,7 +2610,7 @@
     <xf numFmtId="0" fontId="49" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="49" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="49" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="49" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2631,7 +2631,7 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="48" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="48" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2647,7 +2647,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="183" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="64" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2662,7 +2662,7 @@
     <xf numFmtId="1" fontId="54" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="54" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="54" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="54" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2680,7 +2680,7 @@
     <xf numFmtId="0" fontId="64" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="183" fontId="64" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="64" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2698,7 +2698,7 @@
     <xf numFmtId="0" fontId="75" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="183" fontId="48" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="48" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="64" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2710,16 +2710,16 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="48" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="48" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="64" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="64" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="64" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="184" fontId="64" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="64" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="183" fontId="64" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="76" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2741,31 +2741,49 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="49" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="64" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="61" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2779,24 +2797,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="63" fillId="32" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="61" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3763,6 +3763,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -3788,7 +3789,7 @@
       <sheetName val="PPMO_BOQ"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="0"/>
       <sheetData sheetId="1">
         <row r="34">
           <cell r="B34" t="str">
@@ -3801,25 +3802,25 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -4113,75 +4114,75 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M51"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" customWidth="1"/>
     <col min="2" max="2" width="39" customWidth="1"/>
-    <col min="3" max="3" width="11.5546875" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.109375" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" customWidth="1"/>
-    <col min="9" max="9" width="11.109375" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="138" t="s">
+      <c r="A1" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-    </row>
-    <row r="2" spans="1:10" ht="24.6">
-      <c r="A2" s="139" t="s">
+      <c r="B1" s="133"/>
+      <c r="C1" s="133"/>
+      <c r="D1" s="133"/>
+      <c r="E1" s="133"/>
+      <c r="F1" s="133"/>
+      <c r="G1" s="133"/>
+      <c r="H1" s="133"/>
+      <c r="I1" s="133"/>
+      <c r="J1" s="133"/>
+    </row>
+    <row r="2" spans="1:10" ht="25.5">
+      <c r="A2" s="134" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="139"/>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="139"/>
-      <c r="I2" s="139"/>
-      <c r="J2" s="139"/>
-    </row>
-    <row r="3" spans="1:10" ht="18">
-      <c r="A3" s="140" t="s">
+      <c r="B2" s="134"/>
+      <c r="C2" s="134"/>
+      <c r="D2" s="134"/>
+      <c r="E2" s="134"/>
+      <c r="F2" s="134"/>
+      <c r="G2" s="134"/>
+      <c r="H2" s="134"/>
+      <c r="I2" s="134"/>
+      <c r="J2" s="134"/>
+    </row>
+    <row r="3" spans="1:10" ht="18.75">
+      <c r="A3" s="135" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="140"/>
-      <c r="C3" s="140"/>
-      <c r="D3" s="140"/>
-      <c r="E3" s="140"/>
-      <c r="F3" s="140"/>
-      <c r="G3" s="140"/>
-      <c r="H3" s="140"/>
-      <c r="I3" s="140"/>
-      <c r="J3" s="140"/>
+      <c r="B3" s="135"/>
+      <c r="C3" s="135"/>
+      <c r="D3" s="135"/>
+      <c r="E3" s="135"/>
+      <c r="F3" s="135"/>
+      <c r="G3" s="135"/>
+      <c r="H3" s="135"/>
+      <c r="I3" s="135"/>
+      <c r="J3" s="135"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="141" t="s">
+      <c r="A4" s="136" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="141"/>
-      <c r="C4" s="141"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="141"/>
-      <c r="F4" s="141"/>
-      <c r="G4" s="141"/>
-      <c r="H4" s="141"/>
-      <c r="I4" s="141"/>
-      <c r="J4" s="141"/>
+      <c r="B4" s="136"/>
+      <c r="C4" s="136"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="136"/>
+      <c r="F4" s="136"/>
+      <c r="G4" s="136"/>
+      <c r="H4" s="136"/>
+      <c r="I4" s="136"/>
+      <c r="J4" s="136"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="12"/>
@@ -4195,40 +4196,40 @@
       <c r="I5" s="12"/>
       <c r="J5" s="12"/>
     </row>
-    <row r="6" spans="1:10" ht="15.6">
+    <row r="6" spans="1:10" ht="15.75">
       <c r="A6" s="6" t="s">
         <v>52</v>
       </c>
       <c r="B6" s="6"/>
-      <c r="C6" s="142" t="e">
+      <c r="C6" s="137" t="e">
         <f>E51</f>
         <v>#REF!</v>
       </c>
-      <c r="D6" s="143"/>
+      <c r="D6" s="138"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6" t="s">
         <v>53</v>
       </c>
       <c r="H6" s="6"/>
-      <c r="I6" s="142" t="e">
+      <c r="I6" s="137" t="e">
         <f>H51</f>
         <v>#REF!</v>
       </c>
-      <c r="J6" s="143"/>
+      <c r="J6" s="138"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
-      <c r="C7" s="133"/>
-      <c r="D7" s="133"/>
-      <c r="E7" s="133"/>
-      <c r="F7" s="133"/>
-      <c r="H7" s="134"/>
-      <c r="I7" s="134"/>
-      <c r="J7" s="134"/>
-    </row>
-    <row r="8" spans="1:10" ht="16.8">
+      <c r="C7" s="139"/>
+      <c r="D7" s="139"/>
+      <c r="E7" s="139"/>
+      <c r="F7" s="139"/>
+      <c r="H7" s="140"/>
+      <c r="I7" s="140"/>
+      <c r="J7" s="140"/>
+    </row>
+    <row r="8" spans="1:10" ht="16.5">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -4253,32 +4254,32 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="135" t="s">
+      <c r="A10" s="141" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="135" t="s">
+      <c r="B10" s="141" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="137" t="s">
+      <c r="C10" s="143" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="137"/>
-      <c r="E10" s="137"/>
-      <c r="F10" s="137" t="s">
+      <c r="D10" s="143"/>
+      <c r="E10" s="143"/>
+      <c r="F10" s="143" t="s">
         <v>59</v>
       </c>
-      <c r="G10" s="137"/>
-      <c r="H10" s="137"/>
-      <c r="I10" s="135" t="s">
+      <c r="G10" s="143"/>
+      <c r="H10" s="143"/>
+      <c r="I10" s="141" t="s">
         <v>60</v>
       </c>
-      <c r="J10" s="135" t="s">
+      <c r="J10" s="141" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="136"/>
-      <c r="B11" s="136"/>
+      <c r="A11" s="142"/>
+      <c r="B11" s="142"/>
       <c r="C11" s="14" t="s">
         <v>61</v>
       </c>
@@ -4297,10 +4298,10 @@
       <c r="H11" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="I11" s="136"/>
-      <c r="J11" s="136"/>
-    </row>
-    <row r="12" spans="1:10" ht="15.6">
+      <c r="I11" s="142"/>
+      <c r="J11" s="142"/>
+    </row>
+    <row r="12" spans="1:10" ht="15.75">
       <c r="A12" s="22">
         <v>1</v>
       </c>
@@ -4337,7 +4338,7 @@
       </c>
       <c r="J12" s="18"/>
     </row>
-    <row r="13" spans="1:10" ht="15.6">
+    <row r="13" spans="1:10" ht="15.75">
       <c r="A13" s="24"/>
       <c r="B13" s="25"/>
       <c r="C13" s="18"/>
@@ -4349,7 +4350,7 @@
       <c r="I13" s="17"/>
       <c r="J13" s="18"/>
     </row>
-    <row r="14" spans="1:10" ht="31.2">
+    <row r="14" spans="1:10" ht="31.5">
       <c r="A14" s="24">
         <v>2</v>
       </c>
@@ -4386,7 +4387,7 @@
       </c>
       <c r="J14" s="18"/>
     </row>
-    <row r="15" spans="1:10" ht="15.6">
+    <row r="15" spans="1:10" ht="15.75">
       <c r="A15" s="24"/>
       <c r="B15" s="25"/>
       <c r="C15" s="16"/>
@@ -4398,7 +4399,7 @@
       <c r="I15" s="17"/>
       <c r="J15" s="18"/>
     </row>
-    <row r="16" spans="1:10" ht="15.6">
+    <row r="16" spans="1:10" ht="15.75">
       <c r="A16" s="24">
         <v>3</v>
       </c>
@@ -4435,7 +4436,7 @@
       </c>
       <c r="J16" s="18"/>
     </row>
-    <row r="17" spans="1:13" ht="15.6">
+    <row r="17" spans="1:13" ht="15.75">
       <c r="A17" s="24"/>
       <c r="B17" s="27" t="s">
         <v>35</v>
@@ -4455,7 +4456,7 @@
       <c r="I17" s="17"/>
       <c r="J17" s="18"/>
     </row>
-    <row r="18" spans="1:13" ht="15.6">
+    <row r="18" spans="1:13" ht="15.75">
       <c r="A18" s="24"/>
       <c r="B18" s="27"/>
       <c r="C18" s="18"/>
@@ -4467,7 +4468,7 @@
       <c r="I18" s="17"/>
       <c r="J18" s="18"/>
     </row>
-    <row r="19" spans="1:13" ht="15.6">
+    <row r="19" spans="1:13" ht="15.75">
       <c r="A19" s="24">
         <v>4</v>
       </c>
@@ -4505,7 +4506,7 @@
       <c r="J19" s="18"/>
       <c r="M19" s="13"/>
     </row>
-    <row r="20" spans="1:13" ht="15.6">
+    <row r="20" spans="1:13" ht="15.75">
       <c r="A20" s="24"/>
       <c r="B20" s="28" t="s">
         <v>35</v>
@@ -4525,7 +4526,7 @@
       <c r="I20" s="17"/>
       <c r="J20" s="18"/>
     </row>
-    <row r="21" spans="1:13" ht="15.6">
+    <row r="21" spans="1:13" ht="15.75">
       <c r="A21" s="24"/>
       <c r="B21" s="27"/>
       <c r="C21" s="18"/>
@@ -4537,7 +4538,7 @@
       <c r="I21" s="17"/>
       <c r="J21" s="18"/>
     </row>
-    <row r="22" spans="1:13" ht="15.6">
+    <row r="22" spans="1:13" ht="15.75">
       <c r="A22" s="24">
         <v>5</v>
       </c>
@@ -4574,7 +4575,7 @@
       </c>
       <c r="J22" s="18"/>
     </row>
-    <row r="23" spans="1:13" ht="15.6">
+    <row r="23" spans="1:13" ht="15.75">
       <c r="A23" s="24"/>
       <c r="B23" s="28" t="s">
         <v>28</v>
@@ -4594,7 +4595,7 @@
       <c r="I23" s="17"/>
       <c r="J23" s="18"/>
     </row>
-    <row r="24" spans="1:13" ht="15.6">
+    <row r="24" spans="1:13" ht="15.75">
       <c r="A24" s="24"/>
       <c r="B24" s="28" t="s">
         <v>36</v>
@@ -4614,7 +4615,7 @@
       <c r="I24" s="17"/>
       <c r="J24" s="18"/>
     </row>
-    <row r="25" spans="1:13" ht="15.6">
+    <row r="25" spans="1:13" ht="15.75">
       <c r="A25" s="24"/>
       <c r="B25" s="28" t="s">
         <v>29</v>
@@ -4634,7 +4635,7 @@
       <c r="I25" s="17"/>
       <c r="J25" s="18"/>
     </row>
-    <row r="26" spans="1:13" ht="15.6">
+    <row r="26" spans="1:13" ht="15.75">
       <c r="A26" s="24"/>
       <c r="B26" s="28"/>
       <c r="C26" s="18"/>
@@ -4646,7 +4647,7 @@
       <c r="I26" s="17"/>
       <c r="J26" s="18"/>
     </row>
-    <row r="27" spans="1:13" ht="46.8">
+    <row r="27" spans="1:13" ht="31.5">
       <c r="A27" s="24">
         <v>6</v>
       </c>
@@ -4683,7 +4684,7 @@
       </c>
       <c r="J27" s="18"/>
     </row>
-    <row r="28" spans="1:13" ht="15.6">
+    <row r="28" spans="1:13" ht="15.75">
       <c r="A28" s="24"/>
       <c r="B28" s="28" t="s">
         <v>28</v>
@@ -4703,7 +4704,7 @@
       <c r="I28" s="17"/>
       <c r="J28" s="18"/>
     </row>
-    <row r="29" spans="1:13" ht="15.6">
+    <row r="29" spans="1:13" ht="15.75">
       <c r="A29" s="24"/>
       <c r="B29" s="28" t="s">
         <v>30</v>
@@ -4723,7 +4724,7 @@
       <c r="I29" s="17"/>
       <c r="J29" s="18"/>
     </row>
-    <row r="30" spans="1:13" ht="15.6">
+    <row r="30" spans="1:13" ht="15.75">
       <c r="A30" s="24"/>
       <c r="B30" s="28" t="s">
         <v>29</v>
@@ -4743,7 +4744,7 @@
       <c r="I30" s="17"/>
       <c r="J30" s="18"/>
     </row>
-    <row r="31" spans="1:13" ht="15.6">
+    <row r="31" spans="1:13" ht="15.75">
       <c r="A31" s="24"/>
       <c r="B31" s="28"/>
       <c r="C31" s="18"/>
@@ -4755,7 +4756,7 @@
       <c r="I31" s="17"/>
       <c r="J31" s="18"/>
     </row>
-    <row r="32" spans="1:13" ht="15.6">
+    <row r="32" spans="1:13" ht="15.75">
       <c r="A32" s="26">
         <v>7</v>
       </c>
@@ -4792,7 +4793,7 @@
       </c>
       <c r="J32" s="18"/>
     </row>
-    <row r="33" spans="1:10" ht="15.6">
+    <row r="33" spans="1:10" ht="15.75">
       <c r="A33" s="26"/>
       <c r="B33" s="28" t="s">
         <v>28</v>
@@ -4812,7 +4813,7 @@
       <c r="I33" s="17"/>
       <c r="J33" s="18"/>
     </row>
-    <row r="34" spans="1:10" ht="15.6">
+    <row r="34" spans="1:10" ht="15.75">
       <c r="A34" s="24"/>
       <c r="B34" s="28"/>
       <c r="C34" s="18"/>
@@ -4824,7 +4825,7 @@
       <c r="I34" s="17"/>
       <c r="J34" s="18"/>
     </row>
-    <row r="35" spans="1:10" ht="15.6">
+    <row r="35" spans="1:10" ht="15.75">
       <c r="A35" s="24">
         <v>8</v>
       </c>
@@ -4861,7 +4862,7 @@
       </c>
       <c r="J35" s="18"/>
     </row>
-    <row r="36" spans="1:10" ht="15.6">
+    <row r="36" spans="1:10" ht="15.75">
       <c r="A36" s="24"/>
       <c r="B36" s="28" t="s">
         <v>28</v>
@@ -4881,7 +4882,7 @@
       <c r="I36" s="17"/>
       <c r="J36" s="18"/>
     </row>
-    <row r="37" spans="1:10" ht="15.6">
+    <row r="37" spans="1:10" ht="15.75">
       <c r="A37" s="24"/>
       <c r="B37" s="28" t="s">
         <v>29</v>
@@ -4901,7 +4902,7 @@
       <c r="I37" s="17"/>
       <c r="J37" s="18"/>
     </row>
-    <row r="38" spans="1:10" ht="15.6">
+    <row r="38" spans="1:10" ht="15.75">
       <c r="A38" s="26"/>
       <c r="B38" s="28"/>
       <c r="C38" s="18"/>
@@ -4913,7 +4914,7 @@
       <c r="I38" s="17"/>
       <c r="J38" s="18"/>
     </row>
-    <row r="39" spans="1:10" ht="15.6">
+    <row r="39" spans="1:10" ht="15.75">
       <c r="A39" s="24">
         <v>9</v>
       </c>
@@ -4950,7 +4951,7 @@
       </c>
       <c r="J39" s="18"/>
     </row>
-    <row r="40" spans="1:10" ht="15.6">
+    <row r="40" spans="1:10" ht="15.75">
       <c r="A40" s="24"/>
       <c r="B40" s="25"/>
       <c r="C40" s="18"/>
@@ -4962,7 +4963,7 @@
       <c r="I40" s="17"/>
       <c r="J40" s="18"/>
     </row>
-    <row r="41" spans="1:10" ht="15.6">
+    <row r="41" spans="1:10" ht="15.75">
       <c r="A41" s="26">
         <v>10</v>
       </c>
@@ -4999,7 +5000,7 @@
       </c>
       <c r="J41" s="18"/>
     </row>
-    <row r="42" spans="1:10" ht="15.6">
+    <row r="42" spans="1:10" ht="15.75">
       <c r="A42" s="26"/>
       <c r="B42" s="31" t="s">
         <v>47</v>
@@ -5019,7 +5020,7 @@
       <c r="I42" s="17"/>
       <c r="J42" s="18"/>
     </row>
-    <row r="43" spans="1:10" ht="15.6">
+    <row r="43" spans="1:10" ht="15.75">
       <c r="A43" s="26"/>
       <c r="B43" s="30"/>
       <c r="C43" s="18"/>
@@ -5031,7 +5032,7 @@
       <c r="I43" s="17"/>
       <c r="J43" s="18"/>
     </row>
-    <row r="44" spans="1:10" ht="15.6">
+    <row r="44" spans="1:10" ht="15.75">
       <c r="A44" s="26">
         <v>11</v>
       </c>
@@ -5068,7 +5069,7 @@
       </c>
       <c r="J44" s="18"/>
     </row>
-    <row r="45" spans="1:10" ht="15.6">
+    <row r="45" spans="1:10" ht="15.75">
       <c r="A45" s="24"/>
       <c r="B45" s="32" t="s">
         <v>48</v>
@@ -5088,7 +5089,7 @@
       <c r="I45" s="17"/>
       <c r="J45" s="18"/>
     </row>
-    <row r="46" spans="1:10" ht="15.6">
+    <row r="46" spans="1:10" ht="15.75">
       <c r="A46" s="24"/>
       <c r="B46" s="25"/>
       <c r="C46" s="18"/>
@@ -5100,7 +5101,7 @@
       <c r="I46" s="17"/>
       <c r="J46" s="18"/>
     </row>
-    <row r="47" spans="1:10" ht="15.6">
+    <row r="47" spans="1:10" ht="15.75">
       <c r="A47" s="33">
         <v>12</v>
       </c>
@@ -5137,7 +5138,7 @@
       </c>
       <c r="J47" s="18"/>
     </row>
-    <row r="48" spans="1:10" ht="15.6">
+    <row r="48" spans="1:10" ht="15.75">
       <c r="A48" s="22"/>
       <c r="B48" s="35" t="s">
         <v>45</v>
@@ -5157,7 +5158,7 @@
       <c r="I48" s="17"/>
       <c r="J48" s="18"/>
     </row>
-    <row r="49" spans="1:10" ht="15.6">
+    <row r="49" spans="1:10" ht="15.75">
       <c r="A49" s="26"/>
       <c r="B49" s="30"/>
       <c r="C49" s="18"/>
@@ -5169,7 +5170,7 @@
       <c r="I49" s="17"/>
       <c r="J49" s="18"/>
     </row>
-    <row r="50" spans="1:10" ht="15.6">
+    <row r="50" spans="1:10" ht="15.75">
       <c r="A50" s="24">
         <v>12</v>
       </c>
@@ -5203,7 +5204,7 @@
       </c>
       <c r="J50" s="18"/>
     </row>
-    <row r="51" spans="1:10" ht="15.6">
+    <row r="51" spans="1:10" ht="15.75">
       <c r="A51" s="19"/>
       <c r="B51" s="20" t="s">
         <v>64</v>
@@ -5225,12 +5226,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="H7:J7"/>
@@ -5240,6 +5235,12 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I10:I11"/>
     <mergeCell ref="J10:J11"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -5258,17 +5259,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.5546875" customWidth="1"/>
-    <col min="2" max="3" width="13.88671875" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" customWidth="1"/>
+    <col min="2" max="3" width="13.85546875" customWidth="1"/>
     <col min="4" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21">
+    <row r="1" spans="1:8" ht="20.25">
       <c r="A1" s="38">
         <v>152</v>
       </c>
@@ -5282,7 +5283,7 @@
       <c r="G1" s="145"/>
       <c r="H1" s="145"/>
     </row>
-    <row r="2" spans="1:8" ht="15.6">
+    <row r="2" spans="1:8" ht="15.75">
       <c r="A2" s="39" t="s">
         <v>76</v>
       </c>
@@ -5296,7 +5297,7 @@
       <c r="G2" s="147"/>
       <c r="H2" s="147"/>
     </row>
-    <row r="3" spans="1:8" ht="32.4">
+    <row r="3" spans="1:8" ht="31.5">
       <c r="A3" s="40"/>
       <c r="B3" s="41" t="s">
         <v>78</v>
@@ -5320,7 +5321,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="16.8">
+    <row r="4" spans="1:8" ht="17.25">
       <c r="A4" s="40"/>
       <c r="B4" s="148" t="s">
         <v>85</v>
@@ -5343,7 +5344,7 @@
       </c>
       <c r="H4" s="46"/>
     </row>
-    <row r="5" spans="1:8" ht="18">
+    <row r="5" spans="1:8" ht="17.25">
       <c r="A5" s="40"/>
       <c r="B5" s="149"/>
       <c r="C5" s="47" t="s">
@@ -5367,7 +5368,7 @@
         <v>1665</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18">
+    <row r="6" spans="1:8" ht="17.25">
       <c r="A6" s="40"/>
       <c r="B6" s="150" t="s">
         <v>89</v>
@@ -5391,7 +5392,7 @@
       </c>
       <c r="H6" s="46"/>
     </row>
-    <row r="7" spans="1:8" ht="18">
+    <row r="7" spans="1:8" ht="17.25">
       <c r="A7" s="40"/>
       <c r="B7" s="151"/>
       <c r="C7" s="47" t="s">
@@ -5416,7 +5417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="20.399999999999999">
+    <row r="8" spans="1:8" ht="19.5">
       <c r="A8" s="40"/>
       <c r="B8" s="40"/>
       <c r="C8" s="40"/>
@@ -5431,7 +5432,7 @@
         <v>1665</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="20.399999999999999">
+    <row r="9" spans="1:8" ht="19.5">
       <c r="A9" s="40"/>
       <c r="B9" s="40" t="s">
         <v>95</v>
@@ -5448,7 +5449,7 @@
         <v>249.75</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="20.399999999999999">
+    <row r="10" spans="1:8" ht="19.5">
       <c r="A10" s="57"/>
       <c r="B10" s="58">
         <f>+H10</f>
@@ -5473,7 +5474,7 @@
         <v>1914.75</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="16.8">
+    <row r="11" spans="1:8" ht="16.5">
       <c r="A11" s="40"/>
       <c r="B11" s="60">
         <v>10</v>
@@ -5501,18 +5502,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AAC4D04-1B58-42BA-A05B-E669B2EB3EFE}">
   <dimension ref="A1:N12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -5585,12 +5586,12 @@
         <v>7.9244132886315146</v>
       </c>
       <c r="B3" s="116">
-        <f>12.5/3.281</f>
-        <v>3.8098140810728434</v>
+        <f>14.5/3.281</f>
+        <v>4.4193843340444987</v>
       </c>
       <c r="C3" s="116">
-        <f>6/3.281</f>
-        <v>1.8287107589149649</v>
+        <f>5.5/3.281</f>
+        <v>1.6763181956720512</v>
       </c>
       <c r="D3" s="116">
         <v>0.125</v>
@@ -5679,111 +5680,111 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62B3309-9F25-4755-BF2A-62A086A4BBD1}">
   <dimension ref="A1:L84"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="16.8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="4.44140625" style="69" customWidth="1"/>
-    <col min="2" max="2" width="30.5546875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="5.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.44140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="5.44140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.6640625" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="4.42578125" style="69" customWidth="1"/>
+    <col min="2" max="2" width="30.5703125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="5.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="5.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="126" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="127"/>
-      <c r="J1" s="127"/>
-      <c r="K1" s="127"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+      <c r="I1" s="126"/>
+      <c r="J1" s="126"/>
+      <c r="K1" s="126"/>
       <c r="L1" s="106"/>
     </row>
-    <row r="2" spans="1:12" ht="20.399999999999999">
-      <c r="A2" s="128" t="s">
+    <row r="2" spans="1:12" ht="20.25">
+      <c r="A2" s="127" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="128"/>
-      <c r="C2" s="128"/>
-      <c r="D2" s="128"/>
-      <c r="E2" s="128"/>
-      <c r="F2" s="128"/>
-      <c r="G2" s="128"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="128"/>
-      <c r="J2" s="128"/>
-      <c r="K2" s="128"/>
+      <c r="B2" s="127"/>
+      <c r="C2" s="127"/>
+      <c r="D2" s="127"/>
+      <c r="E2" s="127"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="127"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="127"/>
+      <c r="K2" s="127"/>
       <c r="L2" s="113"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="127" t="s">
+      <c r="A3" s="126" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="127"/>
-      <c r="C3" s="127"/>
-      <c r="D3" s="127"/>
-      <c r="E3" s="127"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="127"/>
-      <c r="H3" s="127"/>
-      <c r="I3" s="127"/>
-      <c r="J3" s="127"/>
-      <c r="K3" s="127"/>
+      <c r="B3" s="126"/>
+      <c r="C3" s="126"/>
+      <c r="D3" s="126"/>
+      <c r="E3" s="126"/>
+      <c r="F3" s="126"/>
+      <c r="G3" s="126"/>
+      <c r="H3" s="126"/>
+      <c r="I3" s="126"/>
+      <c r="J3" s="126"/>
+      <c r="K3" s="126"/>
       <c r="L3" s="106"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="129" t="s">
+      <c r="A4" s="128" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="129"/>
-      <c r="C4" s="129"/>
-      <c r="D4" s="129"/>
-      <c r="E4" s="129"/>
-      <c r="F4" s="129"/>
-      <c r="G4" s="129"/>
-      <c r="H4" s="129"/>
-      <c r="I4" s="129"/>
-      <c r="J4" s="129"/>
-      <c r="K4" s="129"/>
-    </row>
-    <row r="5" spans="1:12" ht="21.6">
+      <c r="B4" s="128"/>
+      <c r="C4" s="128"/>
+      <c r="D4" s="128"/>
+      <c r="E4" s="128"/>
+      <c r="F4" s="128"/>
+      <c r="G4" s="128"/>
+      <c r="H4" s="128"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="128"/>
+      <c r="K4" s="128"/>
+    </row>
+    <row r="5" spans="1:12" ht="20.25">
       <c r="A5" s="114" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="J5" s="130" t="s">
+      <c r="J5" s="129" t="s">
         <v>128</v>
       </c>
-      <c r="K5" s="130"/>
+      <c r="K5" s="129"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6" s="131" t="s">
+      <c r="A6" s="124" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="131"/>
-      <c r="C6" s="131"/>
-      <c r="D6" s="131"/>
-      <c r="E6" s="131"/>
-      <c r="F6" s="131"/>
+      <c r="B6" s="124"/>
+      <c r="C6" s="124"/>
+      <c r="D6" s="124"/>
+      <c r="E6" s="124"/>
+      <c r="F6" s="124"/>
       <c r="G6" s="61"/>
-      <c r="H6" s="132" t="s">
-        <v>130</v>
-      </c>
-      <c r="I6" s="132"/>
-      <c r="J6" s="132"/>
-      <c r="K6" s="132"/>
+      <c r="H6" s="125" t="s">
+        <v>136</v>
+      </c>
+      <c r="I6" s="125"/>
+      <c r="J6" s="125"/>
+      <c r="K6" s="125"/>
     </row>
     <row r="7" spans="1:12">
       <c r="B7" s="3"/>
@@ -5848,12 +5849,12 @@
       <c r="J9" s="74"/>
       <c r="K9" s="76"/>
     </row>
-    <row r="10" spans="1:12" ht="30.6">
+    <row r="10" spans="1:12" ht="30.75">
       <c r="A10" s="77">
         <v>1</v>
       </c>
       <c r="B10" s="112" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C10" s="82"/>
       <c r="D10" s="83"/>
@@ -5877,14 +5878,14 @@
       </c>
       <c r="E11" s="83">
         <f>'Size of water tank'!B3+0.15</f>
-        <v>3.9598140810728433</v>
+        <v>4.5693843340444991</v>
       </c>
       <c r="F11" s="84">
         <v>0.3</v>
       </c>
       <c r="G11" s="83">
         <f t="shared" ref="G11" si="0">PRODUCT(C11:F11)</f>
-        <v>9.5919526310174259</v>
+        <v>11.068529276302071</v>
       </c>
       <c r="H11" s="80"/>
       <c r="I11" s="83"/>
@@ -5900,7 +5901,7 @@
       <c r="F12" s="84"/>
       <c r="G12" s="83">
         <f>SUM(G11)</f>
-        <v>9.5919526310174259</v>
+        <v>11.068529276302071</v>
       </c>
       <c r="H12" s="80" t="s">
         <v>24</v>
@@ -5910,7 +5911,7 @@
       </c>
       <c r="J12" s="83">
         <f>G12*I12</f>
-        <v>6915.7978469635636</v>
+        <v>7980.409608213793</v>
       </c>
       <c r="K12" s="81"/>
     </row>
@@ -5927,12 +5928,12 @@
       <c r="J13" s="83"/>
       <c r="K13" s="81"/>
     </row>
-    <row r="14" spans="1:12" ht="30.6">
+    <row r="14" spans="1:12" ht="30.75">
       <c r="A14" s="86">
         <v>2</v>
       </c>
       <c r="B14" s="112" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C14" s="87"/>
       <c r="D14" s="88"/>
@@ -5959,7 +5960,7 @@
       </c>
       <c r="E15" s="88">
         <f>E11</f>
-        <v>3.9598140810728433</v>
+        <v>4.5693843340444991</v>
       </c>
       <c r="F15" s="84">
         <f>'Size of water tank'!H3</f>
@@ -5967,7 +5968,7 @@
       </c>
       <c r="G15" s="88">
         <f>PRODUCT(C15:F15)</f>
-        <v>4.795976315508713</v>
+        <v>5.5342646381510354</v>
       </c>
       <c r="H15" s="84"/>
       <c r="I15" s="88"/>
@@ -5983,7 +5984,7 @@
       <c r="F16" s="84"/>
       <c r="G16" s="88">
         <f>SUM(G15)</f>
-        <v>4.795976315508713</v>
+        <v>5.5342646381510354</v>
       </c>
       <c r="H16" s="84" t="s">
         <v>23</v>
@@ -5993,7 +5994,7 @@
       </c>
       <c r="J16" s="88">
         <f>G16*I16</f>
-        <v>23044.714155782523</v>
+        <v>26592.196928962108</v>
       </c>
       <c r="K16" s="81"/>
     </row>
@@ -6010,7 +6011,7 @@
       <c r="J17" s="83"/>
       <c r="K17" s="81"/>
     </row>
-    <row r="18" spans="1:11" ht="30.6">
+    <row r="18" spans="1:11" ht="30.75">
       <c r="A18" s="77">
         <v>3</v>
       </c>
@@ -6043,7 +6044,7 @@
       </c>
       <c r="E19" s="83">
         <f>E11</f>
-        <v>3.9598140810728433</v>
+        <v>4.5693843340444991</v>
       </c>
       <c r="F19" s="83">
         <f>'Size of water tank'!I3</f>
@@ -6051,7 +6052,7 @@
       </c>
       <c r="G19" s="88">
         <f>PRODUCT(C19:F19)</f>
-        <v>2.3979881577543565</v>
+        <v>2.7671323190755177</v>
       </c>
       <c r="H19" s="80"/>
       <c r="I19" s="83"/>
@@ -6069,7 +6070,7 @@
       <c r="F20" s="83"/>
       <c r="G20" s="83">
         <f>SUM(G19)</f>
-        <v>2.3979881577543565</v>
+        <v>2.7671323190755177</v>
       </c>
       <c r="H20" s="80" t="s">
         <v>24</v>
@@ -6079,7 +6080,7 @@
       </c>
       <c r="J20" s="83">
         <f>G20*I20</f>
-        <v>33438.410147463539</v>
+        <v>38585.889224823884</v>
       </c>
       <c r="K20" s="81"/>
     </row>
@@ -6096,7 +6097,7 @@
       <c r="J21" s="83"/>
       <c r="K21" s="81"/>
     </row>
-    <row r="22" spans="1:11" ht="30.6">
+    <row r="22" spans="1:11" ht="45.75">
       <c r="A22" s="77">
         <v>4</v>
       </c>
@@ -6124,7 +6125,7 @@
       </c>
       <c r="D23" s="88">
         <f>('Size of water tank'!B3-'Size of water tank'!G3*2)+(('Size of water tank'!C3+'Size of water tank'!D3-'Size of water tank'!E3*2)*2)</f>
-        <v>7.5410393172813164</v>
+        <v>7.8458244437671443</v>
       </c>
       <c r="E23" s="83"/>
       <c r="F23" s="83">
@@ -6133,7 +6134,7 @@
       </c>
       <c r="G23" s="88">
         <f>PRODUCT(C23:F23)</f>
-        <v>218.78323945198881</v>
+        <v>227.62577089941712</v>
       </c>
       <c r="H23" s="80"/>
       <c r="I23" s="83"/>
@@ -6149,7 +6150,7 @@
       </c>
       <c r="D24" s="88">
         <f>('Size of water tank'!B3-'Size of water tank'!F3*2+'Size of water tank'!G3*2)+(('Size of water tank'!C3+'Size of water tank'!D3-'Size of water tank'!E3*2)*2)</f>
-        <v>7.2870517118764599</v>
+        <v>7.5918368383622887</v>
       </c>
       <c r="E24" s="83"/>
       <c r="F24" s="83">
@@ -6158,7 +6159,7 @@
       </c>
       <c r="G24" s="88">
         <f t="shared" ref="G24:G32" si="1">PRODUCT(C24:F24)</f>
-        <v>202.41810310767943</v>
+        <v>210.88435662117465</v>
       </c>
       <c r="H24" s="80"/>
       <c r="I24" s="83"/>
@@ -6172,11 +6173,11 @@
       </c>
       <c r="C25" s="87">
         <f>TRUNC(('Size of water tank'!B3-'Size of water tank'!G3*2)/0.15,0)+1-4</f>
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D25" s="88">
         <f>('Size of water tank'!A3-'Size of water tank'!G3*2)+(('Size of water tank'!C3+'Size of water tank'!D3-'Size of water tank'!E3*2)*2)</f>
-        <v>11.655638524839986</v>
+        <v>11.350853398354159</v>
       </c>
       <c r="E25" s="83"/>
       <c r="F25" s="83">
@@ -6185,7 +6186,7 @@
       </c>
       <c r="G25" s="88">
         <f t="shared" si="1"/>
-        <v>151.09161050718501</v>
+        <v>175.16749071534196</v>
       </c>
       <c r="H25" s="80"/>
       <c r="I25" s="83"/>
@@ -6197,11 +6198,11 @@
       <c r="B26" s="90"/>
       <c r="C26" s="87">
         <f>TRUNC(('Size of water tank'!B3-'Size of water tank'!F3*2+'Size of water tank'!G3*2)/0.15,0)+1-4</f>
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D26" s="88">
         <f>('Size of water tank'!A3-'Size of water tank'!F3*2+'Size of water tank'!G3*2)+(('Size of water tank'!C3+'Size of water tank'!D3-'Size of water tank'!E3*2)*2)</f>
-        <v>11.401650919435131</v>
+        <v>11.096865792949304</v>
       </c>
       <c r="E26" s="83"/>
       <c r="F26" s="83">
@@ -6210,7 +6211,7 @@
       </c>
       <c r="G26" s="88">
         <f t="shared" si="1"/>
-        <v>140.76112246216209</v>
+        <v>164.39801174739711</v>
       </c>
       <c r="H26" s="80"/>
       <c r="I26" s="83"/>
@@ -6224,11 +6225,11 @@
       </c>
       <c r="C27" s="82">
         <f>TRUNC(('Size of water tank'!C3-'Size of water tank'!E3)/0.15,0)+1</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D27" s="83">
         <f>('Size of water tank'!A3-'Size of water tank'!G3*2)*2+('Size of water tank'!B3-'Size of water tank'!G3*2)*2</f>
-        <v>23.163669612922888</v>
+        <v>24.382810118866196</v>
       </c>
       <c r="E27" s="83"/>
       <c r="F27" s="83">
@@ -6237,7 +6238,7 @@
       </c>
       <c r="G27" s="88">
         <f t="shared" si="1"/>
-        <v>118.96403159229531</v>
+        <v>115.59258130425457</v>
       </c>
       <c r="H27" s="80"/>
       <c r="I27" s="83"/>
@@ -6249,11 +6250,11 @@
       <c r="B28" s="90"/>
       <c r="C28" s="82">
         <f>TRUNC(('Size of water tank'!C3+'Size of water tank'!E3)/0.15,0)+1</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D28" s="83">
         <f>('Size of water tank'!A3-'Size of water tank'!F3*2+'Size of water tank'!G3*2)*2+('Size of water tank'!B3-'Size of water tank'!F3*2+'Size of water tank'!G3*2)*2</f>
-        <v>22.147719191303466</v>
+        <v>23.366859697246774</v>
       </c>
       <c r="E28" s="83"/>
       <c r="F28" s="83">
@@ -6262,7 +6263,7 @@
       </c>
       <c r="G28" s="88">
         <f t="shared" si="1"/>
-        <v>113.74631090842273</v>
+        <v>110.77622374991061</v>
       </c>
       <c r="H28" s="80"/>
       <c r="I28" s="83"/>
@@ -6301,7 +6302,7 @@
       <c r="B30" s="92"/>
       <c r="C30" s="82">
         <f>2*(TRUNC(((('Size of water tank'!B3-'Size of water tank'!F3*2)+('Size of water tank'!B3-'Size of water tank'!F3*2-'Size of water tank'!M3*2))/2)/0.15,0)+1)-4</f>
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D30" s="83">
         <f>(2*57*('Size of water tank'!J3/1000))+SQRT(('Size of water tank'!M3)^2+('Size of water tank'!N3)^2)</f>
@@ -6314,7 +6315,7 @@
       </c>
       <c r="G30" s="88">
         <f t="shared" si="1"/>
-        <v>20.162049525121002</v>
+        <v>24.406691530409635</v>
       </c>
       <c r="H30" s="80"/>
       <c r="I30" s="83"/>
@@ -6332,7 +6333,7 @@
       </c>
       <c r="D31" s="83">
         <f>(((('Size of water tank'!A3-'Size of water tank'!F3*2)+('Size of water tank'!A3-'Size of water tank'!F3*2-'Size of water tank'!M3*2))/2)+((('Size of water tank'!B3-'Size of water tank'!F3*2)+('Size of water tank'!B3-'Size of water tank'!F3*2-'Size of water tank'!M3*2))/2))*2</f>
-        <v>20.623793558874326</v>
+        <v>21.842934064817637</v>
       </c>
       <c r="E31" s="83"/>
       <c r="F31" s="83">
@@ -6341,7 +6342,7 @@
       </c>
       <c r="G31" s="88">
         <f t="shared" si="1"/>
-        <v>8.1476715294318325</v>
+        <v>8.6293072848662273</v>
       </c>
       <c r="H31" s="80"/>
       <c r="I31" s="83"/>
@@ -6351,14 +6352,14 @@
     <row r="32" spans="1:11">
       <c r="A32" s="77"/>
       <c r="B32" s="92" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C32" s="82">
         <v>6</v>
       </c>
       <c r="D32" s="83">
         <f>F38+0.9</f>
-        <v>2.7287107589149651</v>
+        <v>2.5763181956720511</v>
       </c>
       <c r="E32" s="83"/>
       <c r="F32" s="83">
@@ -6367,7 +6368,7 @@
       </c>
       <c r="G32" s="88">
         <f t="shared" si="1"/>
-        <v>25.872220528971521</v>
+        <v>24.427313262668335</v>
       </c>
       <c r="H32" s="80"/>
       <c r="I32" s="83"/>
@@ -6377,11 +6378,11 @@
     <row r="33" spans="1:11">
       <c r="A33" s="77"/>
       <c r="B33" s="92" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C33" s="82">
         <f>C27</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D33" s="83">
         <f>(4*0.3+0.05*2)</f>
@@ -6394,7 +6395,7 @@
       </c>
       <c r="G33" s="88">
         <f t="shared" ref="G33:G34" si="3">PRODUCT(C33:F33)</f>
-        <v>6.6765432098765434</v>
+        <v>6.162962962962963</v>
       </c>
       <c r="H33" s="80"/>
       <c r="I33" s="83"/>
@@ -6406,7 +6407,7 @@
       <c r="B34" s="92"/>
       <c r="C34" s="82">
         <f>C33</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D34" s="83">
         <f>(4*0.23+0.05*2)</f>
@@ -6419,7 +6420,7 @@
       </c>
       <c r="G34" s="88">
         <f t="shared" si="3"/>
-        <v>5.2385185185185179</v>
+        <v>4.8355555555555556</v>
       </c>
       <c r="H34" s="80"/>
       <c r="I34" s="83"/>
@@ -6435,7 +6436,7 @@
       <c r="F35" s="83"/>
       <c r="G35" s="83">
         <f>SUM(G23:G34)</f>
-        <v>1060.6748044024721</v>
+        <v>1121.719648694778</v>
       </c>
       <c r="H35" s="80" t="s">
         <v>18</v>
@@ -6446,7 +6447,7 @@
       </c>
       <c r="J35" s="93">
         <f>G35*I35</f>
-        <v>142300.13175863566</v>
+        <v>150489.90806889141</v>
       </c>
       <c r="K35" s="81"/>
     </row>
@@ -6463,7 +6464,7 @@
       <c r="J36" s="83"/>
       <c r="K36" s="81"/>
     </row>
-    <row r="37" spans="1:11" ht="30.6">
+    <row r="37" spans="1:11" ht="30.75">
       <c r="A37" s="77">
         <v>5</v>
       </c>
@@ -6490,16 +6491,16 @@
       </c>
       <c r="D38" s="83">
         <f>('Size of water tank'!A3+'Size of water tank'!B3)*2</f>
-        <v>23.468454739408717</v>
+        <v>24.687595245352028</v>
       </c>
       <c r="E38" s="83"/>
       <c r="F38" s="83">
         <f>'Size of water tank'!C3</f>
-        <v>1.8287107589149649</v>
+        <v>1.6763181956720512</v>
       </c>
       <c r="G38" s="83">
         <f>PRODUCT(C38:F38)</f>
-        <v>42.917015677065621</v>
+        <v>41.384265117170422</v>
       </c>
       <c r="H38" s="80"/>
       <c r="I38" s="83"/>
@@ -6514,16 +6515,16 @@
       </c>
       <c r="D39" s="83">
         <f>(('Size of water tank'!A3-'Size of water tank'!F3*2)+('Size of water tank'!B3-'Size of water tank'!F3*2))*2</f>
-        <v>21.842934064817637</v>
+        <v>23.062074570760949</v>
       </c>
       <c r="E39" s="83"/>
       <c r="F39" s="83">
         <f>'Size of water tank'!C3-'Size of water tank'!N3</f>
-        <v>1.5239256324291375</v>
+        <v>1.3715330691862238</v>
       </c>
       <c r="G39" s="83">
         <f t="shared" ref="G39:G40" si="4">PRODUCT(C39:F39)</f>
-        <v>33.287007108835169</v>
+        <v>31.630397917837328</v>
       </c>
       <c r="H39" s="80"/>
       <c r="I39" s="83"/>
@@ -6533,7 +6534,7 @@
     <row r="40" spans="1:11">
       <c r="A40" s="77"/>
       <c r="B40" s="92" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C40" s="82">
         <v>6</v>
@@ -6548,11 +6549,11 @@
       </c>
       <c r="F40" s="83">
         <f>F38</f>
-        <v>1.8287107589149649</v>
+        <v>1.6763181956720512</v>
       </c>
       <c r="G40" s="83">
         <f t="shared" si="4"/>
-        <v>1.3873223691015275</v>
+        <v>1.2717121716764002</v>
       </c>
       <c r="H40" s="80"/>
       <c r="I40" s="83"/>
@@ -6568,7 +6569,7 @@
       <c r="F41" s="83"/>
       <c r="G41" s="83">
         <f>SUM(G38:G40)</f>
-        <v>77.591345155002315</v>
+        <v>74.286375206684141</v>
       </c>
       <c r="H41" s="80" t="s">
         <v>23</v>
@@ -6578,7 +6579,7 @@
       </c>
       <c r="J41" s="83">
         <f>G41*I41</f>
-        <v>74024.471018226861</v>
+        <v>70871.430538432876</v>
       </c>
       <c r="K41" s="81"/>
     </row>
@@ -6595,7 +6596,7 @@
       <c r="J42" s="83"/>
       <c r="K42" s="81"/>
     </row>
-    <row r="43" spans="1:11" ht="30.6">
+    <row r="43" spans="1:11" ht="30.75">
       <c r="A43" s="77">
         <v>6</v>
       </c>
@@ -6615,7 +6616,7 @@
     <row r="44" spans="1:11">
       <c r="A44" s="77"/>
       <c r="B44" s="92" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C44" s="82">
         <v>1</v>
@@ -6626,7 +6627,7 @@
       </c>
       <c r="E44" s="83">
         <f>'Size of water tank'!B3</f>
-        <v>3.8098140810728434</v>
+        <v>4.4193843340444987</v>
       </c>
       <c r="F44" s="83">
         <f>'Size of water tank'!D3</f>
@@ -6634,7 +6635,7 @@
       </c>
       <c r="G44" s="83">
         <f t="shared" ref="G44:G49" si="5">PRODUCT(C44:F44)</f>
-        <v>3.7738176664086378</v>
+        <v>4.3776284930340204</v>
       </c>
       <c r="H44" s="80"/>
       <c r="I44" s="83"/>
@@ -6659,11 +6660,11 @@
       </c>
       <c r="F45" s="83">
         <f>'Size of water tank'!C3</f>
-        <v>1.8287107589149649</v>
+        <v>1.6763181956720512</v>
       </c>
       <c r="G45" s="83">
         <f t="shared" si="5"/>
-        <v>5.0962862538423446</v>
+        <v>4.6715957326888162</v>
       </c>
       <c r="H45" s="80"/>
       <c r="I45" s="83"/>
@@ -6678,7 +6679,7 @@
       </c>
       <c r="D46" s="83">
         <f>'Size of water tank'!B3-'Size of water tank'!F3*2-(14/12/3.281)*2</f>
-        <v>2.692268617291476</v>
+        <v>3.3018388702631314</v>
       </c>
       <c r="E46" s="83">
         <f>'Size of water tank'!F3</f>
@@ -6686,11 +6687,11 @@
       </c>
       <c r="F46" s="83">
         <f>'Size of water tank'!C3</f>
-        <v>1.8287107589149649</v>
+        <v>1.6763181956720512</v>
       </c>
       <c r="G46" s="83">
         <f t="shared" si="5"/>
-        <v>2.0007642329899573</v>
+        <v>2.2492868342575782</v>
       </c>
       <c r="H46" s="80"/>
       <c r="I46" s="83"/>
@@ -6736,7 +6737,7 @@
       </c>
       <c r="D48" s="83">
         <f>(('Size of water tank'!B3-'Size of water tank'!F3*2)+('Size of water tank'!B3-'Size of water tank'!F3*2-'Size of water tank'!M3*2))/2-(14/12/3.281)*3</f>
-        <v>2.0319008432388497</v>
+        <v>2.641471096210505</v>
       </c>
       <c r="E48" s="83">
         <f>'Size of water tank'!M3</f>
@@ -6748,7 +6749,7 @@
       </c>
       <c r="G48" s="83">
         <f t="shared" si="5"/>
-        <v>0.18875134273490163</v>
+        <v>0.24537674555537214</v>
       </c>
       <c r="H48" s="80"/>
       <c r="I48" s="83"/>
@@ -6758,7 +6759,7 @@
     <row r="49" spans="1:11">
       <c r="A49" s="77"/>
       <c r="B49" s="92" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C49" s="82">
         <v>6</v>
@@ -6773,11 +6774,11 @@
       </c>
       <c r="F49" s="83">
         <f>F40-F48</f>
-        <v>1.5239256324291375</v>
+        <v>1.3715330691862238</v>
       </c>
       <c r="G49" s="83">
         <f t="shared" si="5"/>
-        <v>1.156101974251273</v>
+        <v>1.0404917768261457</v>
       </c>
       <c r="H49" s="80"/>
       <c r="I49" s="83"/>
@@ -6795,7 +6796,7 @@
       <c r="F50" s="83"/>
       <c r="G50" s="83">
         <f>SUM(G44:G48)</f>
-        <v>11.630592307748921</v>
+        <v>12.114860617308864</v>
       </c>
       <c r="H50" s="80" t="s">
         <v>24</v>
@@ -6805,7 +6806,7 @@
       </c>
       <c r="J50" s="93">
         <f>G50*I50</f>
-        <v>170451.56403659895</v>
+        <v>177548.7340339392</v>
       </c>
       <c r="K50" s="81"/>
     </row>
@@ -6822,7 +6823,7 @@
       <c r="J51" s="83"/>
       <c r="K51" s="81"/>
     </row>
-    <row r="52" spans="1:11" ht="30.6">
+    <row r="52" spans="1:11" ht="30.75">
       <c r="A52" s="77">
         <v>7</v>
       </c>
@@ -6854,11 +6855,11 @@
       <c r="E53" s="80"/>
       <c r="F53" s="80">
         <f>'Size of water tank'!C3-'Size of water tank'!N3</f>
-        <v>1.5239256324291375</v>
+        <v>1.3715330691862238</v>
       </c>
       <c r="G53" s="83">
         <f t="shared" ref="G53:G55" si="6">PRODUCT(C53:F53)</f>
-        <v>22.91384675398886</v>
+        <v>20.622462078589972</v>
       </c>
       <c r="H53" s="80"/>
       <c r="I53" s="83"/>
@@ -6873,16 +6874,16 @@
       </c>
       <c r="D54" s="80">
         <f>'Size of water tank'!B3-'Size of water tank'!F3*2</f>
-        <v>3.4034339124250734</v>
+        <v>4.0130041653967288</v>
       </c>
       <c r="E54" s="80"/>
       <c r="F54" s="80">
         <f>'Size of water tank'!C3-'Size of water tank'!N3</f>
-        <v>1.5239256324291375</v>
+        <v>1.3715330691862238</v>
       </c>
       <c r="G54" s="83">
         <f t="shared" si="6"/>
-        <v>10.373160354846307</v>
+        <v>11.007935839247352</v>
       </c>
       <c r="H54" s="80"/>
       <c r="I54" s="95"/>
@@ -6899,7 +6900,7 @@
       </c>
       <c r="D55" s="80">
         <f>D47*2+D48*2</f>
-        <v>16.356801788072744</v>
+        <v>17.575942294016052</v>
       </c>
       <c r="E55" s="80"/>
       <c r="F55" s="80">
@@ -6908,7 +6909,7 @@
       </c>
       <c r="G55" s="83">
         <f t="shared" si="6"/>
-        <v>7.0502928758735033</v>
+        <v>7.5757805436404713</v>
       </c>
       <c r="H55" s="80"/>
       <c r="I55" s="95"/>
@@ -6924,7 +6925,7 @@
       <c r="F56" s="84"/>
       <c r="G56" s="83">
         <f>SUM(G53:G55)</f>
-        <v>40.337299984708672</v>
+        <v>39.206178461477798</v>
       </c>
       <c r="H56" s="80" t="s">
         <v>23</v>
@@ -6934,7 +6935,7 @@
       </c>
       <c r="J56" s="83">
         <f>G56*I56</f>
-        <v>17715.738780284202</v>
+        <v>17218.961518496435</v>
       </c>
       <c r="K56" s="81"/>
     </row>
@@ -6951,7 +6952,7 @@
       <c r="J57" s="83"/>
       <c r="K57" s="81"/>
     </row>
-    <row r="58" spans="1:11" ht="30.6">
+    <row r="58" spans="1:11" ht="30.75">
       <c r="A58" s="77">
         <v>8</v>
       </c>
@@ -6982,12 +6983,12 @@
       </c>
       <c r="E59" s="80">
         <f>'Size of water tank'!B3-'Size of water tank'!F3*2-'Size of water tank'!M3*2</f>
-        <v>2.7938636594534185</v>
+        <v>3.4034339124250739</v>
       </c>
       <c r="F59" s="83"/>
       <c r="G59" s="83">
         <f t="shared" ref="G59" si="7">PRODUCT(C59:F59)</f>
-        <v>19.301303346828451</v>
+        <v>23.5124968043183</v>
       </c>
       <c r="H59" s="84"/>
       <c r="I59" s="122"/>
@@ -7003,7 +7004,7 @@
       <c r="F60" s="83"/>
       <c r="G60" s="80">
         <f>SUM(G59:G59)</f>
-        <v>19.301303346828451</v>
+        <v>23.5124968043183</v>
       </c>
       <c r="H60" s="84" t="s">
         <v>23</v>
@@ -7013,7 +7014,7 @@
       </c>
       <c r="J60" s="80">
         <f>G60*I60</f>
-        <v>13969.897336367496</v>
+        <v>17017.874937029497</v>
       </c>
       <c r="K60" s="81"/>
     </row>
@@ -7030,7 +7031,7 @@
       <c r="J61" s="83"/>
       <c r="K61" s="81"/>
     </row>
-    <row r="62" spans="1:11" ht="30.6">
+    <row r="62" spans="1:11" ht="30.75">
       <c r="A62" s="77">
         <v>9</v>
       </c>
@@ -7064,11 +7065,11 @@
       <c r="E63" s="80"/>
       <c r="F63" s="80">
         <f>F53</f>
-        <v>1.5239256324291375</v>
+        <v>1.3715330691862238</v>
       </c>
       <c r="G63" s="83">
         <f>PRODUCT(C63:F63)</f>
-        <v>22.91384675398886</v>
+        <v>20.622462078589972</v>
       </c>
       <c r="H63" s="80"/>
       <c r="I63" s="80"/>
@@ -7084,16 +7085,16 @@
       </c>
       <c r="D64" s="80">
         <f>D54</f>
-        <v>3.4034339124250734</v>
+        <v>4.0130041653967288</v>
       </c>
       <c r="E64" s="80"/>
       <c r="F64" s="80">
         <f>F54</f>
-        <v>1.5239256324291375</v>
+        <v>1.3715330691862238</v>
       </c>
       <c r="G64" s="83">
         <f t="shared" ref="G64:G66" si="8">PRODUCT(C64:F64)</f>
-        <v>10.373160354846307</v>
+        <v>11.007935839247352</v>
       </c>
       <c r="H64" s="80"/>
       <c r="I64" s="80"/>
@@ -7110,7 +7111,7 @@
       </c>
       <c r="D65" s="80">
         <f>D55</f>
-        <v>16.356801788072744</v>
+        <v>17.575942294016052</v>
       </c>
       <c r="E65" s="80"/>
       <c r="F65" s="80">
@@ -7119,7 +7120,7 @@
       </c>
       <c r="G65" s="83">
         <f t="shared" si="8"/>
-        <v>7.0502928758735033</v>
+        <v>7.5757805436404713</v>
       </c>
       <c r="H65" s="80"/>
       <c r="I65" s="80"/>
@@ -7140,12 +7141,12 @@
       </c>
       <c r="E66" s="80">
         <f>E59</f>
-        <v>2.7938636594534185</v>
+        <v>3.4034339124250739</v>
       </c>
       <c r="F66" s="80"/>
       <c r="G66" s="83">
         <f t="shared" si="8"/>
-        <v>19.301303346828451</v>
+        <v>23.5124968043183</v>
       </c>
       <c r="H66" s="80"/>
       <c r="I66" s="80"/>
@@ -7161,7 +7162,7 @@
       <c r="F67" s="80"/>
       <c r="G67" s="80">
         <f>SUM(G63:G66)</f>
-        <v>59.638603331537126</v>
+        <v>62.718675265796094</v>
       </c>
       <c r="H67" s="80" t="s">
         <v>23</v>
@@ -7171,7 +7172,7 @@
       </c>
       <c r="J67" s="80">
         <f>G67*I67</f>
-        <v>18029.942559190305</v>
+        <v>18961.109906355476</v>
       </c>
       <c r="K67" s="81"/>
     </row>
@@ -7188,9 +7189,9 @@
       <c r="J68" s="80"/>
       <c r="K68" s="81"/>
     </row>
-    <row r="69" spans="1:11" ht="30.6">
+    <row r="69" spans="1:11" ht="30.75">
       <c r="A69" s="77">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B69" s="111" t="s">
         <v>112</v>
@@ -7215,13 +7216,13 @@
       </c>
       <c r="D70" s="80">
         <f>G67</f>
-        <v>59.638603331537126</v>
+        <v>62.718675265796094</v>
       </c>
       <c r="E70" s="80"/>
       <c r="F70" s="80"/>
       <c r="G70" s="83">
         <f t="shared" ref="G70" si="9">PRODUCT(C70:F70)</f>
-        <v>59.638603331537126</v>
+        <v>62.718675265796094</v>
       </c>
       <c r="H70" s="80"/>
       <c r="I70" s="80"/>
@@ -7237,7 +7238,7 @@
       <c r="F71" s="80"/>
       <c r="G71" s="80">
         <f>SUM(G70:G70)</f>
-        <v>59.638603331537126</v>
+        <v>62.718675265796094</v>
       </c>
       <c r="H71" s="80" t="s">
         <v>23</v>
@@ -7247,7 +7248,7 @@
       </c>
       <c r="J71" s="80">
         <f>G71*I71</f>
-        <v>27925.77600999226</v>
+        <v>29368.019693209022</v>
       </c>
       <c r="K71" s="81"/>
     </row>
@@ -7264,12 +7265,12 @@
       <c r="J72" s="80"/>
       <c r="K72" s="81"/>
     </row>
-    <row r="73" spans="1:11" ht="31.2">
+    <row r="73" spans="1:11" ht="31.5">
       <c r="A73" s="77">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B73" s="91" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C73" s="82">
         <v>1</v>
@@ -7307,7 +7308,7 @@
     </row>
     <row r="75" spans="1:11" ht="33" customHeight="1">
       <c r="A75" s="77">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B75" s="91" t="s">
         <v>72</v>
@@ -7345,7 +7346,7 @@
       <c r="I76" s="83"/>
       <c r="J76" s="99">
         <f>SUM(J10:J75)</f>
-        <v>533316.44364950538</v>
+        <v>560134.53445835365</v>
       </c>
       <c r="K76" s="100"/>
     </row>
@@ -7367,10 +7368,10 @@
       <c r="B78" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="C78" s="126" t="s">
+      <c r="C78" s="132" t="s">
         <v>66</v>
       </c>
-      <c r="D78" s="126"/>
+      <c r="D78" s="132"/>
       <c r="E78" s="75" t="s">
         <v>67</v>
       </c>
@@ -7386,11 +7387,11 @@
       <c r="B79" s="79" t="s">
         <v>13</v>
       </c>
-      <c r="C79" s="124">
+      <c r="C79" s="130">
         <f>+J76</f>
-        <v>533316.44364950538</v>
-      </c>
-      <c r="D79" s="124"/>
+        <v>560134.53445835365</v>
+      </c>
+      <c r="D79" s="130"/>
       <c r="E79" s="107"/>
       <c r="F79" s="105"/>
       <c r="G79" s="108"/>
@@ -7404,10 +7405,10 @@
       <c r="B80" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="C80" s="124">
+      <c r="C80" s="130">
         <v>500000</v>
       </c>
-      <c r="D80" s="124"/>
+      <c r="D80" s="130"/>
       <c r="E80" s="109">
         <v>100</v>
       </c>
@@ -7423,14 +7424,14 @@
       <c r="B81" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="C81" s="124">
+      <c r="C81" s="130">
         <f>0.95*C80</f>
         <v>475000</v>
       </c>
-      <c r="D81" s="124"/>
+      <c r="D81" s="130"/>
       <c r="E81" s="110">
         <f>C81/C79*100</f>
-        <v>89.06532053456975</v>
+        <v>84.801055956908968</v>
       </c>
       <c r="F81" s="105"/>
       <c r="G81" s="108"/>
@@ -7443,14 +7444,14 @@
       <c r="B82" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="C82" s="124">
+      <c r="C82" s="130">
         <f>C79-C81</f>
-        <v>58316.443649505381</v>
-      </c>
-      <c r="D82" s="124"/>
+        <v>85134.53445835365</v>
+      </c>
+      <c r="D82" s="130"/>
       <c r="E82" s="110">
         <f>C82/C80*100</f>
-        <v>11.663288729901076</v>
+        <v>17.02690689167073</v>
       </c>
       <c r="F82" s="37"/>
     </row>
@@ -7458,11 +7459,11 @@
       <c r="B83" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="C83" s="124">
+      <c r="C83" s="130">
         <f>E83*C80/100</f>
         <v>10000</v>
       </c>
-      <c r="D83" s="124"/>
+      <c r="D83" s="130"/>
       <c r="E83" s="110">
         <v>2</v>
       </c>
@@ -7471,17 +7472,24 @@
       <c r="B84" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="C84" s="125">
+      <c r="C84" s="131">
         <f>E84*C80/100</f>
         <v>15000</v>
       </c>
-      <c r="D84" s="125"/>
+      <c r="D84" s="131"/>
       <c r="E84" s="110">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="C82:D82"/>
+    <mergeCell ref="C83:D83"/>
+    <mergeCell ref="C84:D84"/>
+    <mergeCell ref="C78:D78"/>
+    <mergeCell ref="C79:D79"/>
+    <mergeCell ref="C80:D80"/>
+    <mergeCell ref="C81:D81"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -7489,13 +7497,6 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="J5:K5"/>
-    <mergeCell ref="C82:D82"/>
-    <mergeCell ref="C83:D83"/>
-    <mergeCell ref="C84:D84"/>
-    <mergeCell ref="C78:D78"/>
-    <mergeCell ref="C79:D79"/>
-    <mergeCell ref="C80:D80"/>
-    <mergeCell ref="C81:D81"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.511811023622047" right="0.511811023622047" top="0.39370078740157499" bottom="0.70866141732283505" header="0.31496062992126" footer="0.31496062992126"/>

</xml_diff>